<commit_message>
Changing output: now we have coded_findings and coded_findings_verified
</commit_message>
<xml_diff>
--- a/outputs/errors.xlsx
+++ b/outputs/errors.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>filename</t>
   </si>
@@ -32,6 +32,24 @@
   </si>
   <si>
     <t>timestamp</t>
+  </si>
+  <si>
+    <t>APBREBES (2020) Focus on Plant Variety Protection UPOV Literature Review.pdf</t>
+  </si>
+  <si>
+    <t>CPVR_LEGAL</t>
+  </si>
+  <si>
+    <t>json_parse_failed</t>
+  </si>
+  <si>
+    <t>Invalid control character at: line 1 column 65 (char 64)</t>
+  </si>
+  <si>
+    <t>{"findings":[{"label_code":"IP_FRAMEWORK","snippet":"The move to_x0002_wards stronger intellectual property (IP) protection has been largely driven by external processes, derived from obligations under the World Trade Organization’s (WTO) Agreement on Trade-Related Aspects of Intellectual Property Rights (TRIPS) and the adoption of TRIPS-plus provisions, the latter often medi_x0002_ated via North-South free trade agreements (FTAs).","page_number":4,"reasoning":"Directly discusses CPVR/PVP in relation to TRIPS and TRIPS-plus international IP standards.","confidence":"high"},{"label_code":"IP_FRAMEWORK","snippet":"The WTO’s TRIPS Agreement only requires that WTO members provide for the protection of plant varieties either by patents or by an effec_x0002_tive sui generis system or by any combination thereof, without specifying further what a sui generis system should be. No coun_x0002_try should be forced to establish an IPR regime that goes beyond the minimum requirements of the TRIPS Agreement, including through FTAs obliging countries to join UPOV 1991 or to adopt UPOV-compliant legislation.","page_number":4,"reasoning":"Explicitly links plant variety protection to TRIPS requirements and UPOV-compliant legislation.","confidence":"high"},{"label_code":"IP_FRAMEWORK","snippet":"One conclusion is that the TRIPS Agreement leaves sufficient discretion to governments to de_x0002_sign PVP laws in such a way that the obligations of other trea_x0002_ties are addressed, but that the possibilities for developing countries to implement Farmers’ Rights in their national PVP laws are very restricted once they join UPOV 1991.","page_number":7,"reasoning":"Clearly addresses how PVP laws interact with TRIPS and UPOV frameworks.","confidence":"high"},{"label_code":"IP_FRAMEWORK","snippet":"The study thus recommends that the EU should not push developing countries, especially LDCs, through bilateral agree_x0002_ments to accept far-reaching IP standards (e.g., by requesting adherence to UPOV 1991).","page_number":8,"reasoning"</t>
+  </si>
+  <si>
+    <t>2026-07-02T11:28:16</t>
   </si>
 </sst>
 </file>
@@ -389,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -412,6 +430,26 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
UPdate Page number indication in output
</commit_message>
<xml_diff>
--- a/outputs/errors.xlsx
+++ b/outputs/errors.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>filename</t>
   </si>
@@ -32,6 +32,24 @@
   </si>
   <si>
     <t>timestamp</t>
+  </si>
+  <si>
+    <t>Adelaiye, V.O. (2024) Plant Variety Right and Intellectual Property Law in Nigeria A Review.pdf</t>
+  </si>
+  <si>
+    <t>CPVR_LEGAL</t>
+  </si>
+  <si>
+    <t>json_parse_failed</t>
+  </si>
+  <si>
+    <t>Invalid control character at: line 1 column 5540 (char 5539)</t>
+  </si>
+  <si>
+    <t>{"findings":[{"label_code":"IP_FRAMEWORK","snippet":"One of the most significant developments was the adoption of the International Union for the Protection of New Plant Varieties Convention (UPOV Convention) in 1961. The UPOV system of plant variety protection came into being with the adoption of the International Convention for the Protection of New Varieties of Plants by a Diplomatic Conference in Paris on December 2, 1961. Plant breeding rights was recognized internationally through the Convention, which provides intellectual property protection for breeders and encourage breeders develop new varieties of plant.","reasoning":"This passage directly discusses UPOV and how plant variety rights are recognized within an international IP framework.","confidence":"high"},{"label_code":"IP_FRAMEWORK","snippet":"Meanwhile, the Trade-Related Aspects of Intellectual Property Rights Agreement (TRIPS), which Nigeria is a signatory to, recognizes and provides for the patentability of inventions in all fields of technology and specifically calls for the protection of plant varieties either by patent or by an effective sui generis system or by any combination thereof in line with the provisions of Article 27 of the TRIPS Agreement. Member states of the TRIPS Agreement are obligated to comply with this mandate.","reasoning":"This explicitly refers to TRIPS and its requirement for plant variety protection, fitting the international IP alignment label.","confidence":"high"},{"label_code":"IP_FRAMEWORK","snippet":"The Act aligns with international standards, such as those set by the International Union for the Protection of New Varieties of Plants (UPOV). PVRs grant exclusive rights to breeders of new plant varieties, allowing them to control the propagation and commercialization of their varieties.","reasoning":"This directly states that Nigeria's Act aligns with international standards set by UPOV.","confidence":"high"},{"label_code":"IP_FRAMEWORK","snippet":"In some jurisdiction</t>
+  </si>
+  <si>
+    <t>2026-07-09T13:57:52</t>
   </si>
 </sst>
 </file>
@@ -389,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -412,6 +430,26 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>